<commit_message>
Adminpanel bug report added
</commit_message>
<xml_diff>
--- a/Testcases/Admin Panel.xlsx
+++ b/Testcases/Admin Panel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5d82febcd9738c47/Desktop/Project of sem 8 COPYRIGHT/Testcases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="8_{156BAB73-DD99-4EB7-98B2-662F4F7C1F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80A7833C-55B6-4CBA-84BA-9EE9D2C456DD}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="8_{156BAB73-DD99-4EB7-98B2-662F4F7C1F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC1496DE-340C-4792-B7CC-0CD6FDBE08B3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4A1F185C-2F24-4779-8A1F-00853527109A}"/>
   </bookViews>
@@ -1293,8 +1293,9 @@
   <dimension ref="A1:K47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="64.33203125" customWidth="1"/>
     <col min="4" max="4" width="33.5546875" customWidth="1"/>
     <col min="7" max="7" width="19.5546875" customWidth="1"/>
     <col min="8" max="8" width="29.44140625" customWidth="1"/>

</xml_diff>